<commit_message>
atualizaçao dos resultados de julho
</commit_message>
<xml_diff>
--- a/Resultados GHS - Por semana.xlsx
+++ b/Resultados GHS - Por semana.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/17ab24b3b76d94b1/Desktop/Apresentação de Mídia/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="6" documentId="8_{125821F5-A5F2-4562-970B-E93F06AA5946}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C46E05E6-CCBC-48A2-A729-7D18927FACEF}"/>
+  <xr:revisionPtr revIDLastSave="11" documentId="8_{125821F5-A5F2-4562-970B-E93F06AA5946}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7347B549-48A2-4839-8D91-445277315956}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{33862748-6A9A-4C49-B295-0D4C4EDCD231}"/>
+    <workbookView minimized="1" xWindow="705" yWindow="705" windowWidth="16200" windowHeight="9308" xr2:uid="{33862748-6A9A-4C49-B295-0D4C4EDCD231}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -227,7 +227,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -245,9 +245,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -263,6 +260,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -829,13 +830,15 @@
       <c r="D13" s="6">
         <v>154</v>
       </c>
-      <c r="E13" s="15">
+      <c r="E13" s="6">
         <v>167</v>
       </c>
-      <c r="F13" s="6"/>
+      <c r="F13" s="6">
+        <v>45</v>
+      </c>
       <c r="G13" s="7">
         <f>SUM(B13:F13)</f>
-        <v>609</v>
+        <v>654</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.45">
@@ -851,13 +854,15 @@
       <c r="D14" s="8">
         <v>6914</v>
       </c>
-      <c r="E14" s="16">
+      <c r="E14" s="8">
         <v>6788</v>
       </c>
-      <c r="F14" s="8"/>
+      <c r="F14" s="8">
+        <v>2686</v>
+      </c>
       <c r="G14" s="9">
         <f>SUM(B14:F14)</f>
-        <v>27724</v>
+        <v>30410</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.45">
@@ -876,17 +881,17 @@
         <f t="shared" si="1"/>
         <v>44.896103896103895</v>
       </c>
-      <c r="E15" s="17">
+      <c r="E15" s="10">
         <f t="shared" si="1"/>
         <v>40.646706586826348</v>
       </c>
       <c r="F15" s="10">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>59.68888888888889</v>
       </c>
       <c r="G15" s="9">
         <f t="shared" si="1"/>
-        <v>45.523809523809526</v>
+        <v>46.498470948012233</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.45">
@@ -902,13 +907,15 @@
       <c r="D16" s="6">
         <v>24</v>
       </c>
-      <c r="E16" s="15">
+      <c r="E16" s="6">
         <v>22</v>
       </c>
-      <c r="F16" s="6"/>
+      <c r="F16" s="6">
+        <v>7</v>
+      </c>
       <c r="G16" s="7">
         <f>SUM(B16:F16)</f>
-        <v>78</v>
+        <v>85</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.45">
@@ -924,13 +931,15 @@
       <c r="D17" s="6">
         <v>14</v>
       </c>
-      <c r="E17" s="15">
+      <c r="E17" s="6">
         <v>18</v>
       </c>
-      <c r="F17" s="6"/>
+      <c r="F17" s="6">
+        <v>8</v>
+      </c>
       <c r="G17" s="7">
         <f>SUM(B17:F17)</f>
-        <v>58</v>
+        <v>66</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.45">
@@ -946,13 +955,15 @@
       <c r="D18" s="6">
         <v>2</v>
       </c>
-      <c r="E18" s="15">
+      <c r="E18" s="6">
         <v>3</v>
       </c>
-      <c r="F18" s="6"/>
+      <c r="F18" s="6">
+        <v>2</v>
+      </c>
       <c r="G18" s="7">
         <f>SUM(B18:F18)</f>
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.45">
@@ -1628,27 +1639,27 @@
       </c>
       <c r="B64" s="13">
         <f>G13</f>
-        <v>609</v>
+        <v>654</v>
       </c>
       <c r="C64" s="10">
         <f>G14</f>
-        <v>27724</v>
+        <v>30410</v>
       </c>
       <c r="D64" s="10">
         <f t="shared" si="7"/>
-        <v>45.523809523809526</v>
+        <v>46.498470948012233</v>
       </c>
       <c r="E64" s="13">
         <f>G16</f>
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="F64" s="13">
         <f>G17</f>
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="G64" s="13">
         <f>G18</f>
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="65" spans="1:7" x14ac:dyDescent="0.45">
@@ -1802,27 +1813,27 @@
       </c>
       <c r="B70" s="7">
         <f>SUM(B63:B69)</f>
-        <v>1251</v>
+        <v>1296</v>
       </c>
       <c r="C70" s="9">
         <f>SUM(C63:C69)</f>
-        <v>56509</v>
+        <v>59195</v>
       </c>
       <c r="D70" s="9">
         <f t="shared" si="7"/>
-        <v>45.171063149480418</v>
+        <v>45.675154320987652</v>
       </c>
       <c r="E70" s="7">
         <f>SUM(E63:E69)</f>
-        <v>161</v>
+        <v>168</v>
       </c>
       <c r="F70" s="7">
         <f>SUM(F63:F69)</f>
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="G70" s="7">
         <f>SUM(G63:G69)</f>
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
adicionamos agosto até o S3
</commit_message>
<xml_diff>
--- a/Resultados GHS - Por semana.xlsx
+++ b/Resultados GHS - Por semana.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/17ab24b3b76d94b1/Desktop/Apresentação de Mídia/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11" documentId="8_{125821F5-A5F2-4562-970B-E93F06AA5946}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7347B549-48A2-4839-8D91-445277315956}"/>
+  <xr:revisionPtr revIDLastSave="26" documentId="8_{125821F5-A5F2-4562-970B-E93F06AA5946}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{135048EA-4DA7-4B42-857D-71ACD45B7F0C}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="705" yWindow="705" windowWidth="16200" windowHeight="9308" xr2:uid="{33862748-6A9A-4C49-B295-0D4C4EDCD231}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{33862748-6A9A-4C49-B295-0D4C4EDCD231}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
@@ -993,28 +993,40 @@
       <c r="A21" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B21" s="6"/>
-      <c r="C21" s="6"/>
-      <c r="D21" s="6"/>
+      <c r="B21" s="6">
+        <v>134</v>
+      </c>
+      <c r="C21" s="6">
+        <v>131</v>
+      </c>
+      <c r="D21" s="6">
+        <v>217</v>
+      </c>
       <c r="E21" s="6"/>
       <c r="F21" s="6"/>
       <c r="G21" s="7">
         <f>SUM(B21:F21)</f>
-        <v>0</v>
+        <v>482</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A22" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B22" s="8"/>
-      <c r="C22" s="8"/>
-      <c r="D22" s="8"/>
+      <c r="B22" s="8">
+        <v>6103</v>
+      </c>
+      <c r="C22" s="8">
+        <v>6489</v>
+      </c>
+      <c r="D22" s="8">
+        <v>7091</v>
+      </c>
       <c r="E22" s="8"/>
       <c r="F22" s="8"/>
       <c r="G22" s="9">
         <f>SUM(B22:F22)</f>
-        <v>0</v>
+        <v>19683</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.45">
@@ -1023,15 +1035,15 @@
       </c>
       <c r="B23" s="10">
         <f t="shared" ref="B23:G23" si="2">IFERROR(B22/B21,0)</f>
-        <v>0</v>
+        <v>45.544776119402982</v>
       </c>
       <c r="C23" s="10">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>49.534351145038165</v>
       </c>
       <c r="D23" s="10">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>32.677419354838712</v>
       </c>
       <c r="E23" s="10">
         <f t="shared" si="2"/>
@@ -1043,49 +1055,67 @@
       </c>
       <c r="G23" s="9">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>40.836099585062243</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A24" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B24" s="6"/>
-      <c r="C24" s="6"/>
-      <c r="D24" s="6"/>
+      <c r="B24" s="6">
+        <v>14</v>
+      </c>
+      <c r="C24" s="6">
+        <v>23</v>
+      </c>
+      <c r="D24" s="6">
+        <v>25</v>
+      </c>
       <c r="E24" s="6"/>
       <c r="F24" s="6"/>
       <c r="G24" s="7">
         <f>SUM(B24:F24)</f>
-        <v>0</v>
+        <v>62</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A25" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B25" s="6"/>
-      <c r="C25" s="6"/>
-      <c r="D25" s="6"/>
+      <c r="B25" s="6">
+        <v>11</v>
+      </c>
+      <c r="C25" s="6">
+        <v>19</v>
+      </c>
+      <c r="D25" s="6">
+        <v>12</v>
+      </c>
       <c r="E25" s="6"/>
       <c r="F25" s="6"/>
       <c r="G25" s="7">
         <f>SUM(B25:F25)</f>
-        <v>0</v>
+        <v>42</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A26" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="B26" s="6"/>
-      <c r="C26" s="6"/>
-      <c r="D26" s="6"/>
+      <c r="B26" s="6">
+        <v>2</v>
+      </c>
+      <c r="C26" s="6">
+        <v>0</v>
+      </c>
+      <c r="D26" s="6">
+        <v>2</v>
+      </c>
       <c r="E26" s="6"/>
       <c r="F26" s="6"/>
       <c r="G26" s="7">
         <f>SUM(B26:F26)</f>
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.45">
@@ -1668,27 +1698,27 @@
       </c>
       <c r="B65" s="13">
         <f>G21</f>
-        <v>0</v>
+        <v>482</v>
       </c>
       <c r="C65" s="10">
         <f>G22</f>
-        <v>0</v>
+        <v>19683</v>
       </c>
       <c r="D65" s="10">
         <f t="shared" si="7"/>
-        <v>0</v>
+        <v>40.836099585062243</v>
       </c>
       <c r="E65" s="13">
         <f>G24</f>
-        <v>0</v>
+        <v>62</v>
       </c>
       <c r="F65" s="13">
         <f>G25</f>
-        <v>0</v>
+        <v>42</v>
       </c>
       <c r="G65" s="13">
         <f>G26</f>
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="66" spans="1:7" x14ac:dyDescent="0.45">
@@ -1813,27 +1843,27 @@
       </c>
       <c r="B70" s="7">
         <f>SUM(B63:B69)</f>
-        <v>1296</v>
+        <v>1778</v>
       </c>
       <c r="C70" s="9">
         <f>SUM(C63:C69)</f>
-        <v>59195</v>
+        <v>78878</v>
       </c>
       <c r="D70" s="9">
         <f t="shared" si="7"/>
-        <v>45.675154320987652</v>
+        <v>44.363329583802027</v>
       </c>
       <c r="E70" s="7">
         <f>SUM(E63:E69)</f>
-        <v>168</v>
+        <v>230</v>
       </c>
       <c r="F70" s="7">
         <f>SUM(F63:F69)</f>
-        <v>126</v>
+        <v>168</v>
       </c>
       <c r="G70" s="7">
         <f>SUM(G63:G69)</f>
-        <v>12</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>